<commit_message>
Выставка: добавлена Marie Claire Beauty Group (Cegedis, ABO, France Lab)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VLjCgLaLytKuq4s5CCcueg
</commit_message>
<xml_diff>
--- a/exhibition/contacts.xlsx
+++ b/exhibition/contacts.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Стенд INPD (Китай)" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Контакты!$A$1:$W$22</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Контакты!$A$1:$W$23</definedName>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Стенд INPD (Китай)'!$A$1:$D$43</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="559" uniqueCount="395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="404">
   <si>
     <t xml:space="preserve">№</t>
   </si>
@@ -1012,6 +1012,33 @@
   </si>
   <si>
     <t xml:space="preserve">photos/018_ms_beautilab_card.jpg ; photos/018b_ms_beautilab_stand.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Регион Иль-де-Франс (запад от Парижа: Гервиль / Мант-ля-Жоли — ABO); France Lab — Париж, хаб в Нью-Йорке</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marie Claire Beauty Group: CEGEDIS (парфюм) + ABO Cosmétiques (косметика) + France Lab (разработка) + Decortiat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cosmetic 360, стенд DB28 (Innovation Route — Formulation)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Полный цикл от создания бренда до производства, под ключ или по этапам: ПАРФЮМ (CEGEDIS — производство парфюмерии), уход, макияж, уход за волосами, ароматы для дома (ABO — производство и фасовка селективной, органической и натуральной косметики, в т.ч. парфюмерной воды). France Lab — разработка ароматов и косметики на заказ, дизайн упаковки, регуляторика. Новинка на стенде: парфюм нового поколения — без спирта, на водной основе, стойкий. На витрине: парфюмы, кремы, палетки теней, румяна, помады</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Производитель парфюма</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Группа принадлежит медиагруппе Marie Claire. France Lab куплена в 2015 г., ABO Cosmétiques и Cegedis — в 2018 г., дизайн-агентство Desdoigts &amp; Associés — в 2020 г. Вместе закрывают цепочку от создания бренда до производства. Decortiat — в источниках не найден (возможно, партнёр/подразделение).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.premiumbeautynews.com/en/marie-claire-group-to-speed-up,14015 ; https://beautymatter.com/articles/marie-claire-group-continues-diversification-in-beauty-sector ; https://www.cosmetic-valley.com/en/annuaire-entreprises/abo-cosmetiques ; https://www.premiumbeautynews.com/en/france-lab-sets-up-offices-and-an,9839 ; https://www.cbnews.fr/medias/groupe-marie-claire-rachete-agence-desdoigts-associes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Взять контакт на стенде DB28; запросить: парфюм (в т.ч. безспиртовой на водной основе), MOQ, сроки, цены; продукты для губ и макияж</t>
+  </si>
+  <si>
+    <t xml:space="preserve">photos/022_marie_claire_beauty_group.jpg</t>
   </si>
   <si>
     <t xml:space="preserve">Мейссак (Коррез), Новая Аквитания; второй сайт — Юссак</t>
@@ -2341,7 +2368,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:W22"/>
+  <dimension ref="A1:W23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -3431,7 +3458,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
@@ -3448,11 +3475,9 @@
         <v>254</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G18" s="4" t="s">
         <v>255</v>
       </c>
+      <c r="G18" s="2"/>
       <c r="H18" s="2"/>
       <c r="I18" s="2" t="s">
         <v>256</v>
@@ -3463,27 +3488,31 @@
       <c r="M18" s="2"/>
       <c r="N18" s="2"/>
       <c r="O18" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="P18" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q18" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="P18" s="2" t="s">
+      <c r="R18" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="Q18" s="2"/>
-      <c r="R18" s="2" t="s">
+      <c r="S18" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="S18" s="2" t="s">
+      <c r="T18" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="T18" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="U18" s="2"/>
+      <c r="U18" s="2" t="s">
+        <v>58</v>
+      </c>
       <c r="V18" s="2" t="s">
         <v>42</v>
       </c>
       <c r="W18" s="2" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3497,20 +3526,20 @@
         <v>45</v>
       </c>
       <c r="D19" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="E19" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="F19" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G19" s="4" t="s">
         <v>264</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>265</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>266</v>
       </c>
       <c r="H19" s="2"/>
       <c r="I19" s="2" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
@@ -3518,202 +3547,257 @@
       <c r="M19" s="2"/>
       <c r="N19" s="2"/>
       <c r="O19" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="P19" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="Q19" s="2"/>
+      <c r="R19" s="2" t="s">
         <v>268</v>
       </c>
-      <c r="P19" s="2" t="s">
+      <c r="S19" s="2" t="s">
         <v>269</v>
       </c>
-      <c r="Q19" s="2" t="s">
+      <c r="T19" s="2" t="s">
         <v>270</v>
-      </c>
-      <c r="R19" s="2" t="s">
-        <v>271</v>
-      </c>
-      <c r="S19" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="T19" s="2" t="s">
-        <v>273</v>
       </c>
       <c r="U19" s="2"/>
       <c r="V19" s="2" t="s">
         <v>42</v>
       </c>
       <c r="W19" s="2" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="n">
         <v>19</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>275</v>
+        <v>143</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>45</v>
       </c>
       <c r="D20" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2" t="s">
         <v>276</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>277</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>278</v>
-      </c>
-      <c r="G20" s="2"/>
-      <c r="H20" s="4" t="s">
-        <v>279</v>
-      </c>
-      <c r="I20" s="2" t="s">
-        <v>280</v>
       </c>
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
-      <c r="L20" s="2" t="s">
-        <v>281</v>
-      </c>
+      <c r="L20" s="2"/>
       <c r="M20" s="2"/>
       <c r="N20" s="2"/>
       <c r="O20" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="P20" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="Q20" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="R20" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="S20" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="T20" s="2" t="s">
         <v>282</v>
-      </c>
-      <c r="P20" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q20" s="2" t="s">
-        <v>283</v>
-      </c>
-      <c r="R20" s="2" t="s">
-        <v>284</v>
-      </c>
-      <c r="S20" s="2" t="s">
-        <v>285</v>
-      </c>
-      <c r="T20" s="2" t="s">
-        <v>286</v>
       </c>
       <c r="U20" s="2"/>
       <c r="V20" s="2" t="s">
         <v>42</v>
       </c>
       <c r="W20" s="2" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="n">
         <v>20</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>275</v>
+        <v>284</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D21" s="2"/>
+      <c r="D21" s="2" t="s">
+        <v>285</v>
+      </c>
       <c r="E21" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="G21" s="2"/>
+      <c r="H21" s="4" t="s">
         <v>288</v>
       </c>
-      <c r="F21" s="2" t="s">
+      <c r="I21" s="2" t="s">
         <v>289</v>
-      </c>
-      <c r="G21" s="2"/>
-      <c r="H21" s="2"/>
-      <c r="I21" s="2" t="s">
-        <v>290</v>
       </c>
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
-      <c r="L21" s="2"/>
+      <c r="L21" s="2" t="s">
+        <v>290</v>
+      </c>
       <c r="M21" s="2"/>
       <c r="N21" s="2"/>
-      <c r="O21" s="2"/>
+      <c r="O21" s="2" t="s">
+        <v>291</v>
+      </c>
       <c r="P21" s="2" t="s">
         <v>67</v>
       </c>
       <c r="Q21" s="2" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="R21" s="2" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="S21" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="T21" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="U21" s="2"/>
       <c r="V21" s="2" t="s">
         <v>42</v>
       </c>
       <c r="W21" s="2" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="n">
         <v>21</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>296</v>
+        <v>284</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D22" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="F22" s="2" t="s">
         <v>298</v>
       </c>
-      <c r="F22" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G22" s="4" t="s">
+      <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2" t="s">
         <v>299</v>
-      </c>
-      <c r="H22" s="4" t="s">
-        <v>300</v>
-      </c>
-      <c r="I22" s="2" t="s">
-        <v>301</v>
       </c>
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
       <c r="M22" s="2"/>
       <c r="N22" s="2"/>
-      <c r="O22" s="2" t="s">
+      <c r="O22" s="2"/>
+      <c r="P22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q22" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="R22" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="S22" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="P22" s="2" t="s">
+      <c r="T22" s="2" t="s">
         <v>303</v>
-      </c>
-      <c r="Q22" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="R22" s="2" t="s">
-        <v>305</v>
-      </c>
-      <c r="S22" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="T22" s="2" t="s">
-        <v>307</v>
       </c>
       <c r="U22" s="2"/>
       <c r="V22" s="2" t="s">
         <v>42</v>
       </c>
       <c r="W22" s="2" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G23" s="4" t="s">
         <v>308</v>
       </c>
+      <c r="H23" s="4" t="s">
+        <v>309</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="J23" s="2"/>
+      <c r="K23" s="2"/>
+      <c r="L23" s="2"/>
+      <c r="M23" s="2"/>
+      <c r="N23" s="2"/>
+      <c r="O23" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="P23" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="Q23" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="R23" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="S23" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="T23" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="U23" s="2"/>
+      <c r="V23" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="W23" s="2" t="s">
+        <v>317</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W22"/>
+  <autoFilter ref="A1:W23"/>
   <hyperlinks>
     <hyperlink ref="G2" r:id="rId1" display="https://www.dachser.fr"/>
     <hyperlink ref="H2" r:id="rId2" display="https://www.dachser.com/en/cosmetic-logistics"/>
@@ -3731,10 +3815,10 @@
     <hyperlink ref="G13" r:id="rId14" display="www.effervescence-lab.com"/>
     <hyperlink ref="G15" r:id="rId15" display="https://www.laboratoiresbea.com"/>
     <hyperlink ref="G17" r:id="rId16" display="https://www.msbeautilab.com"/>
-    <hyperlink ref="G18" r:id="rId17" display="https://simah-cosmetiques.fr"/>
-    <hyperlink ref="H20" r:id="rId18" display="https://welcon.kocca.kr/en/directory/company/cosplan-inc--5601"/>
-    <hyperlink ref="G22" r:id="rId19" display="https://iwasecosfa.eu"/>
-    <hyperlink ref="H22" r:id="rId20" display="https://iwasecosfa-eu.covalo.com/"/>
+    <hyperlink ref="G19" r:id="rId17" display="https://simah-cosmetiques.fr"/>
+    <hyperlink ref="H21" r:id="rId18" display="https://welcon.kocca.kr/en/directory/company/cosplan-inc--5601"/>
+    <hyperlink ref="G23" r:id="rId19" display="https://iwasecosfa.eu"/>
+    <hyperlink ref="H23" r:id="rId20" display="https://iwasecosfa-eu.covalo.com/"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3765,10 +3849,10 @@
         <v>1</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>309</v>
+        <v>318</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>310</v>
+        <v>319</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3776,11 +3860,11 @@
         <v>23</v>
       </c>
       <c r="B2" s="6" t="n">
-        <f aca="false">COUNTIF(Контакты!$B$2:$B$22,A2)</f>
+        <f aca="false">COUNTIF(Контакты!$B$2:$B$23,A2)</f>
         <v>1</v>
       </c>
       <c r="C2" s="6" t="n">
-        <f aca="false">COUNTIFS(Контакты!$B$2:$B$22,A2,Контакты!$U$2:$U$22,"Высокий")</f>
+        <f aca="false">COUNTIFS(Контакты!$B$2:$B$23,A2,Контакты!$U$2:$U$23,"Высокий")</f>
         <v>0</v>
       </c>
     </row>
@@ -3789,11 +3873,11 @@
         <v>44</v>
       </c>
       <c r="B3" s="6" t="n">
-        <f aca="false">COUNTIF(Контакты!$B$2:$B$22,A3)</f>
+        <f aca="false">COUNTIF(Контакты!$B$2:$B$23,A3)</f>
         <v>6</v>
       </c>
       <c r="C3" s="6" t="n">
-        <f aca="false">COUNTIFS(Контакты!$B$2:$B$22,A3,Контакты!$U$2:$U$22,"Высокий")</f>
+        <f aca="false">COUNTIFS(Контакты!$B$2:$B$23,A3,Контакты!$U$2:$U$23,"Высокий")</f>
         <v>4</v>
       </c>
     </row>
@@ -3802,11 +3886,11 @@
         <v>131</v>
       </c>
       <c r="B4" s="6" t="n">
-        <f aca="false">COUNTIF(Контакты!$B$2:$B$22,A4)</f>
+        <f aca="false">COUNTIF(Контакты!$B$2:$B$23,A4)</f>
         <v>1</v>
       </c>
       <c r="C4" s="6" t="n">
-        <f aca="false">COUNTIFS(Контакты!$B$2:$B$22,A4,Контакты!$U$2:$U$22,"Высокий")</f>
+        <f aca="false">COUNTIFS(Контакты!$B$2:$B$23,A4,Контакты!$U$2:$U$23,"Высокий")</f>
         <v>0</v>
       </c>
     </row>
@@ -3815,51 +3899,51 @@
         <v>143</v>
       </c>
       <c r="B5" s="6" t="n">
-        <f aca="false">COUNTIF(Контакты!$B$2:$B$22,A5)</f>
-        <v>10</v>
+        <f aca="false">COUNTIF(Контакты!$B$2:$B$23,A5)</f>
+        <v>11</v>
       </c>
       <c r="C5" s="6" t="n">
-        <f aca="false">COUNTIFS(Контакты!$B$2:$B$22,A5,Контакты!$U$2:$U$22,"Высокий")</f>
-        <v>3</v>
+        <f aca="false">COUNTIFS(Контакты!$B$2:$B$23,A5,Контакты!$U$2:$U$23,"Высокий")</f>
+        <v>4</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>275</v>
+        <v>284</v>
       </c>
       <c r="B6" s="6" t="n">
-        <f aca="false">COUNTIF(Контакты!$B$2:$B$22,A6)</f>
+        <f aca="false">COUNTIF(Контакты!$B$2:$B$23,A6)</f>
         <v>2</v>
       </c>
       <c r="C6" s="6" t="n">
-        <f aca="false">COUNTIFS(Контакты!$B$2:$B$22,A6,Контакты!$U$2:$U$22,"Высокий")</f>
+        <f aca="false">COUNTIFS(Контакты!$B$2:$B$23,A6,Контакты!$U$2:$U$23,"Высокий")</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>296</v>
+        <v>305</v>
       </c>
       <c r="B7" s="6" t="n">
-        <f aca="false">COUNTIF(Контакты!$B$2:$B$22,A7)</f>
+        <f aca="false">COUNTIF(Контакты!$B$2:$B$23,A7)</f>
         <v>1</v>
       </c>
       <c r="C7" s="6" t="n">
-        <f aca="false">COUNTIFS(Контакты!$B$2:$B$22,A7,Контакты!$U$2:$U$22,"Высокий")</f>
+        <f aca="false">COUNTIFS(Контакты!$B$2:$B$23,A7,Контакты!$U$2:$U$23,"Высокий")</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>311</v>
+        <v>320</v>
       </c>
       <c r="B8" s="7" t="n">
         <f aca="false">SUM(B2:B7)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C8" s="7" t="n">
         <f aca="false">SUM(C2:C7)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3872,7 +3956,7 @@
         <v>2</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>309</v>
+        <v>318</v>
       </c>
       <c r="C10" s="6"/>
     </row>
@@ -3881,7 +3965,7 @@
         <v>132</v>
       </c>
       <c r="B11" s="6" t="n">
-        <f aca="false">COUNTIF(Контакты!$C$2:$C$22,A11)</f>
+        <f aca="false">COUNTIF(Контакты!$C$2:$C$23,A11)</f>
         <v>1</v>
       </c>
       <c r="C11" s="6"/>
@@ -3891,8 +3975,8 @@
         <v>45</v>
       </c>
       <c r="B12" s="6" t="n">
-        <f aca="false">COUNTIF(Контакты!$C$2:$C$22,A12)</f>
-        <v>11</v>
+        <f aca="false">COUNTIF(Контакты!$C$2:$C$23,A12)</f>
+        <v>12</v>
       </c>
       <c r="C12" s="6"/>
     </row>
@@ -3901,7 +3985,7 @@
         <v>24</v>
       </c>
       <c r="B13" s="6" t="n">
-        <f aca="false">COUNTIF(Контакты!$C$2:$C$22,A13)</f>
+        <f aca="false">COUNTIF(Контакты!$C$2:$C$23,A13)</f>
         <v>1</v>
       </c>
       <c r="C13" s="6"/>
@@ -3911,7 +3995,7 @@
         <v>186</v>
       </c>
       <c r="B14" s="6" t="n">
-        <f aca="false">COUNTIF(Контакты!$C$2:$C$22,A14)</f>
+        <f aca="false">COUNTIF(Контакты!$C$2:$C$23,A14)</f>
         <v>1</v>
       </c>
       <c r="C14" s="6"/>
@@ -3921,7 +4005,7 @@
         <v>60</v>
       </c>
       <c r="B15" s="6" t="n">
-        <f aca="false">COUNTIF(Контакты!$C$2:$C$22,A15)</f>
+        <f aca="false">COUNTIF(Контакты!$C$2:$C$23,A15)</f>
         <v>3</v>
       </c>
       <c r="C15" s="6"/>
@@ -3931,7 +4015,7 @@
         <v>72</v>
       </c>
       <c r="B16" s="6" t="n">
-        <f aca="false">COUNTIF(Контакты!$C$2:$C$22,A16)</f>
+        <f aca="false">COUNTIF(Контакты!$C$2:$C$23,A16)</f>
         <v>4</v>
       </c>
       <c r="C16" s="6"/>
@@ -3966,585 +4050,585 @@
         <v>4</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>312</v>
+        <v>321</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>313</v>
+        <v>322</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>314</v>
+        <v>323</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>315</v>
+        <v>324</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>316</v>
+        <v>325</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>317</v>
+        <v>326</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>318</v>
+        <v>327</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>319</v>
+        <v>328</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>316</v>
+        <v>325</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>320</v>
+        <v>329</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>318</v>
+        <v>327</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>321</v>
+        <v>330</v>
       </c>
       <c r="B4" s="9" t="s">
         <v>60</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>324</v>
+        <v>333</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>325</v>
+        <v>334</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>326</v>
+        <v>335</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>327</v>
+        <v>336</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>328</v>
+        <v>337</v>
       </c>
       <c r="B6" s="9" t="s">
         <v>60</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>329</v>
+        <v>338</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>331</v>
+        <v>340</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>60</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>332</v>
+        <v>341</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="B8" s="9" t="s">
         <v>60</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>334</v>
+        <v>343</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>318</v>
+        <v>327</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>335</v>
+        <v>344</v>
       </c>
       <c r="B9" s="9" t="s">
         <v>60</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>336</v>
+        <v>345</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>318</v>
+        <v>327</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>337</v>
+        <v>346</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="C10" s="9" t="s">
+        <v>348</v>
+      </c>
+      <c r="D10" s="9" t="s">
         <v>339</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>330</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>340</v>
+        <v>349</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>341</v>
+        <v>350</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>343</v>
+        <v>352</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>344</v>
+        <v>353</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>345</v>
+        <v>354</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>346</v>
+        <v>355</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>347</v>
+        <v>356</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>348</v>
+        <v>357</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>349</v>
+        <v>358</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>350</v>
+        <v>359</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>351</v>
+        <v>360</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>352</v>
+        <v>361</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>353</v>
+        <v>362</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>318</v>
+        <v>327</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>354</v>
+        <v>363</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>355</v>
+        <v>364</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>356</v>
+        <v>365</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>357</v>
+        <v>366</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>358</v>
+        <v>367</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>357</v>
+        <v>366</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>359</v>
+        <v>368</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>360</v>
+        <v>369</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>318</v>
+        <v>327</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>361</v>
+        <v>370</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>362</v>
+        <v>371</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>363</v>
+        <v>372</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>364</v>
+        <v>373</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>318</v>
+        <v>327</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>365</v>
+        <v>374</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>355</v>
+        <v>364</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>366</v>
+        <v>375</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>367</v>
+        <v>376</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="s">
-        <v>368</v>
+        <v>377</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>357</v>
+        <v>366</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="s">
-        <v>369</v>
+        <v>378</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>370</v>
+        <v>379</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>371</v>
+        <v>380</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>372</v>
+        <v>381</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="8" t="s">
-        <v>373</v>
+        <v>382</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>374</v>
+        <v>383</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="8" t="s">
-        <v>375</v>
+        <v>384</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>376</v>
+        <v>385</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>318</v>
+        <v>327</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="8" t="s">
-        <v>377</v>
+        <v>386</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>378</v>
+        <v>387</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>318</v>
+        <v>327</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="9" t="s">
-        <v>379</v>
+        <v>388</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>380</v>
+        <v>389</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="9" t="s">
-        <v>381</v>
+        <v>390</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>357</v>
+        <v>366</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="9" t="s">
-        <v>382</v>
+        <v>391</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>383</v>
+        <v>392</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="9" t="s">
-        <v>384</v>
+        <v>393</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>325</v>
+        <v>334</v>
       </c>
       <c r="C35" s="9"/>
       <c r="D35" s="9" t="s">
-        <v>385</v>
+        <v>394</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="8" t="s">
-        <v>386</v>
+        <v>395</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>325</v>
+        <v>334</v>
       </c>
       <c r="C36" s="9"/>
       <c r="D36" s="9" t="s">
-        <v>385</v>
+        <v>394</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="8" t="s">
-        <v>387</v>
+        <v>396</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>325</v>
+        <v>334</v>
       </c>
       <c r="C37" s="9"/>
       <c r="D37" s="9" t="s">
-        <v>385</v>
+        <v>394</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="9" t="s">
-        <v>388</v>
+        <v>397</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>325</v>
+        <v>334</v>
       </c>
       <c r="C38" s="9"/>
       <c r="D38" s="9" t="s">
-        <v>385</v>
+        <v>394</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="9" t="s">
-        <v>389</v>
+        <v>398</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>325</v>
+        <v>334</v>
       </c>
       <c r="C39" s="9"/>
       <c r="D39" s="9" t="s">
-        <v>385</v>
+        <v>394</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="8" t="s">
-        <v>390</v>
+        <v>399</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>325</v>
+        <v>334</v>
       </c>
       <c r="C40" s="9"/>
       <c r="D40" s="9" t="s">
-        <v>385</v>
+        <v>394</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="9" t="s">
-        <v>391</v>
+        <v>400</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>325</v>
+        <v>334</v>
       </c>
       <c r="C41" s="9"/>
       <c r="D41" s="9" t="s">
-        <v>385</v>
+        <v>394</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="9" t="s">
-        <v>392</v>
+        <v>401</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>325</v>
+        <v>334</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>393</v>
+        <v>402</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>385</v>
+        <v>394</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="8" t="s">
-        <v>394</v>
+        <v>403</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>325</v>
+        <v>334</v>
       </c>
       <c r="C43" s="9"/>
       <c r="D43" s="9" t="s">
-        <v>385</v>
+        <v>394</v>
       </c>
     </row>
   </sheetData>

</xml_diff>